<commit_message>
Net Tú and Việt out instead of routing them through Chi
Both fronted more for the BBQ than their shortfall, so collecting 862.274
from them only to send most of it straight back was churn. Now only Quỳnh,
Hà and Hiếu pay in, and Chi banks Tú and Việt the difference — 237.726 and
137.726. Chi still nets 2.211.370, and the two BBQ advances moved into the
parameter block so the BBQ line and the refunds read from the same cells.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017FddK1NHADf37yURgGtMXU
</commit_message>
<xml_diff>
--- a/group-travel-split/chia-tien-chuyen-di.xlsx
+++ b/group-travel-split/chia-tien-chuyen-di.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,12 +75,6 @@
       <b val="1"/>
       <color rgb="001F3B4D"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="000000FF"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -169,7 +163,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="10" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -535,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -659,6 +653,14 @@
       </c>
       <c r="E6" s="11" t="n"/>
       <c r="F6" s="11" t="n"/>
+      <c r="H6" s="8" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Tú ứng trả bữa BBQ</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -680,6 +682,14 @@
       </c>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="n"/>
+      <c r="H7" s="8" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Việt ứng trả bữa BBQ</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -750,12 +760,13 @@
           <t>Ăn tối BBQ</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
-        <v>2100000</v>
+      <c r="B11" s="10">
+        <f>$H$6+$H$7</f>
+        <v/>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Tú 1.100.000 · Việt 1.000.000</t>
+          <t>Tú và Việt ứng trả</t>
         </is>
       </c>
       <c r="D11" s="10">
@@ -867,7 +878,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Mọi người đóng cho Chi, Chi bank lại phần đã ứng cho Việt &amp; Tú.</t>
+          <t>Tú và Việt không phải đóng — tiền hai bạn ứng đang dư.</t>
         </is>
       </c>
     </row>
@@ -881,6 +892,11 @@
         <f>$F$15</f>
         <v/>
       </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>phần còn thiếu</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -892,6 +908,11 @@
         <f>$F$15</f>
         <v/>
       </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>phần còn thiếu</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -903,72 +924,57 @@
         <f>$F$15</f>
         <v/>
       </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>phần còn thiếu</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Việt  →  Chi</t>
-        </is>
-      </c>
-      <c r="B22" s="19">
-        <f>$F$15</f>
-        <v/>
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Chi  →  Tú</t>
+        </is>
+      </c>
+      <c r="B22" s="20">
+        <f>$H$6-$F$15</f>
+        <v/>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>đã ứng 1.100.000 cho BBQ → đang dư, nhận lại phần chênh</t>
+        </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Tú  →  Chi</t>
-        </is>
-      </c>
-      <c r="B23" s="19">
-        <f>$F$15</f>
-        <v/>
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Chi  →  Việt</t>
+        </is>
+      </c>
+      <c r="B23" s="20">
+        <f>$H$7-$F$15</f>
+        <v/>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>đã ứng 1.000.000 cho BBQ → đang dư, nhận lại phần chênh</t>
+        </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>Chi  →  Tú</t>
-        </is>
-      </c>
-      <c r="B24" s="20" t="n">
-        <v>1100000</v>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>hoàn lại tiền đã ứng trả bữa BBQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>Chi  →  Việt</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>hoàn lại tiền đã ứng trả bữa BBQ</t>
-        </is>
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Chi thực nhận</t>
+        </is>
+      </c>
+      <c r="B24" s="16">
+        <f>SUM(B19:B21)-SUM(B22:B23)</f>
+        <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>Chi thực nhận</t>
-        </is>
-      </c>
-      <c r="B26" s="16">
-        <f>SUM(B19:B23)-SUM(B24:B25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Giả định: tiền cọc gom thành quỹ chung do Chi giữ và Chi dùng để thanh toán. Nếu cọc nộp cho bên khác thì cách chốt sẽ khác.</t>
         </is>

</xml_diff>